<commit_message>
lol I did most of the results
</commit_message>
<xml_diff>
--- a/05_Manuscript/results/3_factor.xlsx
+++ b/05_Manuscript/results/3_factor.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -388,13 +388,13 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>-0.05790242382169856</v>
+        <v>-0.06091770730429641</v>
       </c>
       <c r="B2">
-        <v>0.9561537499761388</v>
+        <v>0.9550291766436688</v>
       </c>
       <c r="C2">
-        <v>-0.05258470193760166</v>
+        <v>-0.03999307959895881</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -414,13 +414,13 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>-0.003205041153705154</v>
+        <v>-0.002681095393081495</v>
       </c>
       <c r="B3">
-        <v>0.9196704489553269</v>
+        <v>0.9187933350583621</v>
       </c>
       <c r="C3">
-        <v>-0.01099970350954209</v>
+        <v>-0.01375669621951984</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -440,13 +440,13 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>-0.04645993743002346</v>
+        <v>-0.05036243313769261</v>
       </c>
       <c r="B4">
-        <v>0.9187337819674486</v>
+        <v>0.9182567307130645</v>
       </c>
       <c r="C4">
-        <v>-0.0007808709797371325</v>
+        <v>0.01355994670554626</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -466,13 +466,13 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>0.03191587792127767</v>
+        <v>0.03095860127430147</v>
       </c>
       <c r="B5">
-        <v>0.851171455968062</v>
+        <v>0.8509584222932678</v>
       </c>
       <c r="C5">
-        <v>-0.01775110819820049</v>
+        <v>-0.01541034583948538</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -492,13 +492,13 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>-0.07202300090870134</v>
+        <v>-0.07184949191707403</v>
       </c>
       <c r="B6">
-        <v>0.821196201346835</v>
+        <v>0.8231755152841801</v>
       </c>
       <c r="C6">
-        <v>0.09326787517953065</v>
+        <v>0.08612501824313404</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -518,13 +518,13 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>0.07600731124792134</v>
+        <v>0.07232538604239891</v>
       </c>
       <c r="B7">
-        <v>0.7812931028642377</v>
+        <v>0.7810112348834245</v>
       </c>
       <c r="C7">
-        <v>0.0008338894877161548</v>
+        <v>0.01445650066147252</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -544,13 +544,13 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>0.1356260097971541</v>
+        <v>0.137132703653939</v>
       </c>
       <c r="B8">
-        <v>0.7409779963439695</v>
+        <v>0.7424655406618001</v>
       </c>
       <c r="C8">
-        <v>0.05249975144950311</v>
+        <v>0.0404607595003298</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -570,13 +570,13 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>0.1634663265830723</v>
+        <v>0.1681033909166523</v>
       </c>
       <c r="B9">
-        <v>0.620075796976874</v>
+        <v>0.6224597479914296</v>
       </c>
       <c r="C9">
-        <v>0.0874866830169658</v>
+        <v>0.06003062313381157</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -596,13 +596,13 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>0.08155512145522155</v>
+        <v>0.08079442108111384</v>
       </c>
       <c r="B10">
-        <v>0.511323983420479</v>
+        <v>0.5109588868268095</v>
       </c>
       <c r="C10">
-        <v>0.0008875297942968664</v>
+        <v>0.003140438771026508</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -622,13 +622,13 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>0.2020917580022664</v>
+        <v>0.2035385473727707</v>
       </c>
       <c r="B11">
-        <v>0.4862269269416017</v>
+        <v>0.4846258213780952</v>
       </c>
       <c r="C11">
-        <v>-0.1117553588278552</v>
+        <v>-0.1146051140501545</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -648,39 +648,39 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>0.05637744784486842</v>
+        <v>0.2215826764889385</v>
       </c>
       <c r="B12">
-        <v>0.4422721019535271</v>
+        <v>0.3522838806238748</v>
       </c>
       <c r="C12">
-        <v>0.336041022044966</v>
+        <v>0.1185289717317063</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Q4_17</t>
+          <t>Q4_13</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Parts of me are immortal.</t>
+          <t>The most important parts of me are immaterial and lasting.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>0.2187196074556324</v>
+        <v>0.5069412164700892</v>
       </c>
       <c r="B13">
-        <v>0.3482958038633376</v>
+        <v>0.2495783032392657</v>
       </c>
       <c r="C13">
-        <v>0.1418076187539197</v>
+        <v>0.04733195366131049</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -689,24 +689,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Q4_13</t>
+          <t>Q5_4</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The most important parts of me are immaterial and lasting.</t>
+          <t>My beliefs and values have been shared with others who will carry them.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>0.5071355432652683</v>
+        <v>0.485021231279749</v>
       </c>
       <c r="B14">
-        <v>0.2468832307421739</v>
+        <v>0.2457788243469955</v>
       </c>
       <c r="C14">
-        <v>0.05187265042959</v>
+        <v>0.1249010428936522</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -715,24 +715,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Q5_4</t>
+          <t>Q5_19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>My beliefs and values have been shared with others who will carry them.</t>
+          <t>I consider myself a part of something bigger which will last forever.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>0.4870162624583443</v>
+        <v>0.5564133838401571</v>
       </c>
       <c r="B15">
-        <v>0.2428984519297805</v>
+        <v>0.2271516049224381</v>
       </c>
       <c r="C15">
-        <v>0.1242733305172612</v>
+        <v>-0.1137742721152704</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -741,24 +741,24 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Q5_19</t>
+          <t>Q4_6</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>I consider myself a part of something bigger which will last forever.</t>
+          <t>I have cared for people and things which will last a long time.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>0.5564712100424521</v>
+        <v>-0.06600374466264708</v>
       </c>
       <c r="B16">
-        <v>0.228865289262442</v>
+        <v>0.1931165129504992</v>
       </c>
       <c r="C16">
-        <v>-0.1179190387596582</v>
+        <v>0.5540480663043553</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -767,24 +767,24 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Q4_6</t>
+          <t>Q5_12</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>I have cared for people and things which will last a long time.</t>
+          <t>I don't entirely believe I will die.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>-0.06146511755806489</v>
+        <v>0.4966825890032878</v>
       </c>
       <c r="B17">
-        <v>0.178970648601886</v>
+        <v>0.1413787846292117</v>
       </c>
       <c r="C17">
-        <v>0.5703293883290352</v>
+        <v>-0.06913493617537395</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -793,24 +793,24 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Q5_12</t>
+          <t>Q2_19</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>I don't entirely believe I will die.</t>
+          <t>I am comforted by knowing my loved ones will live on after me.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>0.5000217523078037</v>
+        <v>0.4762382834535538</v>
       </c>
       <c r="B18">
-        <v>0.1433401407878846</v>
+        <v>0.1343515479181815</v>
       </c>
       <c r="C18">
-        <v>-0.08816950678243378</v>
+        <v>0.1143892333151447</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -819,24 +819,24 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Q2_19</t>
+          <t>Q5_17</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>I am comforted by knowing my loved ones will live on after me.</t>
+          <t>I am comforted by the fact that my genes can/will be carried on in the future.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>0.4826284184320306</v>
+        <v>0.5939743434918814</v>
       </c>
       <c r="B19">
-        <v>0.1329160332853294</v>
+        <v>0.1321100129227104</v>
       </c>
       <c r="C19">
-        <v>0.09012534173859714</v>
+        <v>0.1910320759070989</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -845,24 +845,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Q5_17</t>
+          <t>Q4_9</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>I am comforted by the fact that my genes can/will be carried on in the future.</t>
+          <t>I believe the effects of my life will continue after I am gone.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>0.5308140348232574</v>
+        <v>0.5218632648593625</v>
       </c>
       <c r="B20">
-        <v>0.1286715692873443</v>
+        <v>0.1305072625022746</v>
       </c>
       <c r="C20">
-        <v>0.1842792217862475</v>
+        <v>0.2184053708327927</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -882,13 +882,13 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>0.5980256370143668</v>
+        <v>0.3857560138721186</v>
       </c>
       <c r="B21">
-        <v>0.1277317663247002</v>
+        <v>0.129931774162943</v>
       </c>
       <c r="C21">
-        <v>0.1837810111460815</v>
+        <v>0.2318333526689904</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -897,24 +897,24 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Q4_9</t>
+          <t>Q5_6</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>I believe the effects of my life will continue after I am gone.</t>
+          <t>My beliefs and values will exist in the future more than most people's.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>0.3911837317655451</v>
+        <v>0.4599590785717924</v>
       </c>
       <c r="B22">
-        <v>0.12550088171708</v>
+        <v>0.11525241466913</v>
       </c>
       <c r="C22">
-        <v>0.2191050884601715</v>
+        <v>0.2010341525353974</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -923,24 +923,24 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Q5_6</t>
+          <t>Q4_4</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>My beliefs and values will exist in the future more than most people's.</t>
+          <t>I have lived a life exemplifying timeless virtues.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>0.4642063871173375</v>
+        <v>0.01291689336817368</v>
       </c>
       <c r="B23">
-        <v>0.1106337473797514</v>
+        <v>0.1086122234534972</v>
       </c>
       <c r="C23">
-        <v>0.1954551929081698</v>
+        <v>0.4233231587251129</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -949,24 +949,24 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Q4_4</t>
+          <t>Q2_13</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>I have lived a life exemplifying timeless virtues.</t>
+          <t>I believe I will be reincarnated.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>0.534924548564864</v>
+        <v>0.5355486693046458</v>
       </c>
       <c r="B24">
-        <v>0.1061348456296252</v>
+        <v>0.1038446708037436</v>
       </c>
       <c r="C24">
-        <v>-0.1757379058158396</v>
+        <v>-0.1719936778133148</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -986,13 +986,13 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>0.0193376544544687</v>
+        <v>0.6019998996364664</v>
       </c>
       <c r="B25">
-        <v>0.09976172467627915</v>
+        <v>0.09836924711680738</v>
       </c>
       <c r="C25">
-        <v>0.4184913087949647</v>
+        <v>-0.02128637515955923</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1001,24 +1001,24 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Q2_13</t>
+          <t>Q5_15</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>I believe I will be reincarnated.</t>
+          <t>My personality will live on in others.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>0.6014990467967871</v>
+        <v>0.7147862234808784</v>
       </c>
       <c r="B26">
-        <v>0.09746449672689711</v>
+        <v>0.09641052890875768</v>
       </c>
       <c r="C26">
-        <v>-0.01910581705296876</v>
+        <v>-0.1113789688553787</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1027,24 +1027,24 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Q5_15</t>
+          <t>Q2_4</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>My personality will live on in others.</t>
+          <t>I feel I have taken part in something bigger than myself.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>0.7127545768787207</v>
+        <v>0.6456936711289843</v>
       </c>
       <c r="B27">
-        <v>0.09694309207076839</v>
+        <v>0.0770206997462048</v>
       </c>
       <c r="C27">
-        <v>-0.1061277749349883</v>
+        <v>-0.09525012570218772</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1053,24 +1053,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Q2_4</t>
+          <t>Q4_15</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>I feel I have taken part in something bigger than myself.</t>
+          <t>There are many things I can do to leave my mark on the world.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>0.6451382533275548</v>
+        <v>-0.05204604291382586</v>
       </c>
       <c r="B28">
-        <v>0.07745918722315771</v>
+        <v>0.06923260375742397</v>
       </c>
       <c r="C28">
-        <v>-0.0944893133481307</v>
+        <v>0.6570944675370111</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1079,24 +1079,24 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Q4_15</t>
+          <t>Q4_18</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>There are many things I can do to leave my mark on the world.</t>
+          <t>I believe will not die.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>0.6879640238873882</v>
+        <v>0.6815698985457778</v>
       </c>
       <c r="B29">
-        <v>0.06230862388560841</v>
+        <v>0.06259077379575956</v>
       </c>
       <c r="C29">
-        <v>0.08879419493254084</v>
+        <v>0.1148018796786372</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1116,13 +1116,13 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>-0.04809219225368286</v>
+        <v>-0.02078005130751248</v>
       </c>
       <c r="B30">
-        <v>0.05167685637988469</v>
+        <v>0.04883041113069248</v>
       </c>
       <c r="C30">
-        <v>0.6846192179482197</v>
+        <v>0.5078306945417739</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1131,24 +1131,24 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Q4_18</t>
+          <t>Q4_11</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>I believe will not die.</t>
+          <t>I have a hard time believing I will physically die.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>-0.01302923891954362</v>
+        <v>0.679931853081178</v>
       </c>
       <c r="B31">
-        <v>0.03708672602813715</v>
+        <v>0.03504275823456241</v>
       </c>
       <c r="C31">
-        <v>0.5043639402505881</v>
+        <v>-0.1210579540461681</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1157,24 +1157,24 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Q4_11</t>
+          <t>Q2_9</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>I have a hard time believing I will physically die.</t>
+          <t>Through my interactions with them, others have picked up parts of my personality.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>0.675952448924565</v>
+        <v>0.2662577572737167</v>
       </c>
       <c r="B32">
-        <v>0.03473992930687556</v>
+        <v>0.01504553972659767</v>
       </c>
       <c r="C32">
-        <v>-0.1083959119764895</v>
+        <v>0.3380622982001329</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1183,24 +1183,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Q2_9</t>
+          <t>Q4_8</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Through my interactions with them, others have picked up parts of my personality.</t>
+          <t>I have children or students which take after me.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>0.6825851905511834</v>
+        <v>0.677172993879231</v>
       </c>
       <c r="B33">
-        <v>0.009014238933694071</v>
+        <v>0.01353444029050219</v>
       </c>
       <c r="C33">
-        <v>0.2450646486538571</v>
+        <v>0.2573482953989928</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1220,13 +1220,13 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>0.6910185709293754</v>
+        <v>0.6958626123779098</v>
       </c>
       <c r="B34">
-        <v>0.007955958909992024</v>
+        <v>0.008690525589193072</v>
       </c>
       <c r="C34">
-        <v>-0.1168126925298588</v>
+        <v>-0.1335101564499569</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1246,13 +1246,13 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>0.2700474035603814</v>
+        <v>0.7382558042600756</v>
       </c>
       <c r="B35">
-        <v>0.00748075471171395</v>
+        <v>-0.008559353687979636</v>
       </c>
       <c r="C35">
-        <v>0.3409846860768721</v>
+        <v>0.03012902788342076</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1261,24 +1261,24 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Q4_8</t>
+          <t>Q5_9</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>I have children or students which take after me.</t>
+          <t>I have contributed to things which will be meaningful.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>0.7397074072686407</v>
+        <v>0.7336333079149185</v>
       </c>
       <c r="B36">
-        <v>-0.00998849955415336</v>
+        <v>-0.02737522064314158</v>
       </c>
       <c r="C36">
-        <v>0.02770298118095238</v>
+        <v>-0.0715918839262611</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1287,24 +1287,24 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Q5_9</t>
+          <t>Q4_1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>I have contributed to things which will be meaningful.</t>
+          <t>Others would say I have impacted their lives.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>0.6281928712713564</v>
+        <v>0.6233859256586911</v>
       </c>
       <c r="B37">
-        <v>-0.02558749611784661</v>
+        <v>-0.02813701263275868</v>
       </c>
       <c r="C37">
-        <v>-0.08226030522898778</v>
+        <v>-0.05829502009029467</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1324,13 +1324,13 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>0.7322669271734952</v>
+        <v>0.4100487965125535</v>
       </c>
       <c r="B38">
-        <v>-0.02775518552264179</v>
+        <v>-0.02892339925054528</v>
       </c>
       <c r="C38">
-        <v>-0.0674048464185573</v>
+        <v>3.671522645023538E-05</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1339,24 +1339,24 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Q4_1</t>
+          <t>Q4_12</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Others would say I have impacted their lives.</t>
+          <t>Life is long enough for me to do what I find meaningful.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>0.4134838213409465</v>
+        <v>0.7828454660339774</v>
       </c>
       <c r="B39">
-        <v>-0.02806290456854028</v>
+        <v>-0.03726722923256573</v>
       </c>
       <c r="C39">
-        <v>-0.01540370668144157</v>
+        <v>-0.04812728208254484</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1365,24 +1365,24 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Q4_12</t>
+          <t>Q2_16</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Life is long enough for me to do what I find meaningful.</t>
+          <t>I have taken part in activities or events which will impact the future.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>0.7826295121565822</v>
+        <v>0.529020798923874</v>
       </c>
       <c r="B40">
-        <v>-0.03856252557603152</v>
+        <v>-0.03821310541581132</v>
       </c>
       <c r="C40">
-        <v>-0.04651902760441429</v>
+        <v>0.2157624340170954</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1391,24 +1391,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Q2_16</t>
+          <t>Q5_7</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>I have taken part in activities or events which will impact the future.</t>
+          <t>I have helped transmit ideas from the past to the future.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>0.5292182159567081</v>
+        <v>0.6051161099420329</v>
       </c>
       <c r="B41">
-        <v>-0.04495946806713604</v>
+        <v>-0.04537822265228384</v>
       </c>
       <c r="C41">
-        <v>0.2314439595389449</v>
+        <v>0.01444023114934977</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1417,24 +1417,24 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Q5_7</t>
+          <t>Q4_2</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>I have helped transmit ideas from the past to the future.</t>
+          <t>I have lived a life which will be looked at with approval.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>0.6074584557764557</v>
+        <v>0.664894573660978</v>
       </c>
       <c r="B42">
-        <v>-0.04550849470294208</v>
+        <v>-0.04707628517807665</v>
       </c>
       <c r="C42">
-        <v>0.006072190978356732</v>
+        <v>-0.01397174459165542</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1443,24 +1443,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Q4_2</t>
+          <t>Q2_15</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>I have lived a life which will be looked at with approval.</t>
+          <t>I have taken part in organizations which impact the future.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>0.7513341931141495</v>
+        <v>0.7529011322514187</v>
       </c>
       <c r="B43">
-        <v>-0.04981944248666071</v>
+        <v>-0.04773275053258542</v>
       </c>
       <c r="C43">
-        <v>-0.02305076997954511</v>
+        <v>-0.03291155974582914</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1480,13 +1480,13 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>0.6623618793382795</v>
+        <v>0.6978710851235959</v>
       </c>
       <c r="B44">
-        <v>-0.05020129641329881</v>
+        <v>-0.05613123186029861</v>
       </c>
       <c r="C44">
-        <v>0.001660918422742524</v>
+        <v>0.1976537527705832</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1495,24 +1495,24 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Q2_15</t>
+          <t>Q2_2</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>I have taken part in organizations which impact the future.</t>
+          <t>I have contributed to the world in a unique way.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>0.7454099578581752</v>
+        <v>0.7409264038246699</v>
       </c>
       <c r="B45">
-        <v>-0.05829252778599878</v>
+        <v>-0.06164645475260721</v>
       </c>
       <c r="C45">
-        <v>-0.1115061235585456</v>
+        <v>-0.0869061424296642</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1532,13 +1532,13 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>0.7036556167471306</v>
+        <v>0.6778010038680595</v>
       </c>
       <c r="B46">
-        <v>-0.05973972452605161</v>
+        <v>-0.07206213946308032</v>
       </c>
       <c r="C46">
-        <v>0.1818230931138825</v>
+        <v>-0.1193643505000708</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1547,24 +1547,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Q2_2</t>
+          <t>Q2_20</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>I have contributed to the world in a unique way.</t>
+          <t>I have imparted knowledge and skills on to others.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>0.67382746854779</v>
+        <v>0.6085185804963759</v>
       </c>
       <c r="B47">
-        <v>-0.07226308507699157</v>
+        <v>-0.08036840522216378</v>
       </c>
       <c r="C47">
-        <v>-0.1055460728544043</v>
+        <v>0.2138695848414034</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1573,24 +1573,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Q2_20</t>
+          <t>Q4_5</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>I have imparted knowledge and skills on to others.</t>
+          <t>I have created things which will last a long time.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>0.6102666325778581</v>
+        <v>0.180734803573338</v>
       </c>
       <c r="B48">
-        <v>-0.08626629223584382</v>
+        <v>-0.1930982775211019</v>
       </c>
       <c r="C48">
-        <v>0.221647852348959</v>
+        <v>0.4580073550778012</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1599,36 +1599,10 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Q4_5</t>
+          <t>Q4_7</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
-        <is>
-          <t>I have created things which will last a long time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49">
-        <v>0.1914613162493777</v>
-      </c>
-      <c r="B49">
-        <v>-0.1992421159297743</v>
-      </c>
-      <c r="C49">
-        <v>0.4309394108496338</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Q4_7</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
         <is>
           <t>I have already accomplished what I want to in life.</t>
         </is>

</xml_diff>